<commit_message>
LESSON 16 -DB Design -HuongGiang 20.06.2025
</commit_message>
<xml_diff>
--- a/Java24 HuongGiang Database Design.xlsx
+++ b/Java24 HuongGiang Database Design.xlsx
@@ -1,13 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\java24\3. Database\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{770D3CEB-3101-486E-BB8F-61DB3C5B9D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="B1 Thiet ke" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,8 +24,121 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
+  <si>
+    <t>MatHang</t>
+  </si>
+  <si>
+    <t>MaMH</t>
+  </si>
+  <si>
+    <t>TenMH</t>
+  </si>
+  <si>
+    <t>KichThuoc(s)</t>
+  </si>
+  <si>
+    <t>GiaBan</t>
+  </si>
+  <si>
+    <t>LoaiMatHang</t>
+  </si>
+  <si>
+    <t>ChatLieu(s)</t>
+  </si>
+  <si>
+    <t>MauSac(s)</t>
+  </si>
+  <si>
+    <t>HinhAnh(s)</t>
+  </si>
+  <si>
+    <t>DonHang</t>
+  </si>
+  <si>
+    <t>MaDH</t>
+  </si>
+  <si>
+    <t>MaKH</t>
+  </si>
+  <si>
+    <t>NgayDat</t>
+  </si>
+  <si>
+    <t>DiaChi</t>
+  </si>
+  <si>
+    <t>SDT</t>
+  </si>
+  <si>
+    <t>HinhThucTT</t>
+  </si>
+  <si>
+    <t>SoLuong</t>
+  </si>
+  <si>
+    <t>TongTien</t>
+  </si>
+  <si>
+    <t>PhiVanChuyen</t>
+  </si>
+  <si>
+    <t>TrangThai</t>
+  </si>
+  <si>
+    <t>KhachHang</t>
+  </si>
+  <si>
+    <t>HoTen</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>MatKHau</t>
+  </si>
+  <si>
+    <t>Diachi</t>
+  </si>
+  <si>
+    <t>DangNhapMXH</t>
+  </si>
+  <si>
+    <t>LSTrangThaiDH</t>
+  </si>
+  <si>
+    <t>MaLS</t>
+  </si>
+  <si>
+    <t>NguoiPhuTrach</t>
+  </si>
+  <si>
+    <t>NgayCapNhat</t>
+  </si>
+  <si>
+    <t>MaLoai</t>
+  </si>
+  <si>
+    <t>TenLoai</t>
+  </si>
+  <si>
+    <t>HinhAnhSP</t>
+  </si>
+  <si>
+    <t>MaSP</t>
+  </si>
+  <si>
+    <t>URL</t>
+  </si>
+  <si>
+    <t>ThanhToan</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -29,15 +148,21 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +170,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +476,265 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B5:M16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="13" width="15.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B5" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+    </row>
+    <row r="6" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+    </row>
+    <row r="7" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B7" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+    </row>
+    <row r="8" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+    </row>
+    <row r="9" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B9" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+    </row>
+    <row r="10" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B10" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+    </row>
+    <row r="11" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B11" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+    </row>
+    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+    </row>
+    <row r="13" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+    </row>
+    <row r="14" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B14" s="2"/>
+      <c r="C14" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+    </row>
+    <row r="15" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B15" s="2"/>
+      <c r="C15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.35">
+      <c r="B16" s="2"/>
+      <c r="C16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>